<commit_message>
feat(samples): add MCA course admission sample files for both RPA bot and allocation engine
</commit_message>
<xml_diff>
--- a/docs/sample_data/admission_sample.xlsx
+++ b/docs/sample_data/admission_sample.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,17 +478,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Priya Sharma</t>
+          <t>Aarav Sharma</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>priya.sharma@student.edu</t>
+          <t>aarav.sharma@student.smartuniversity.edu</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>9876543210</t>
+          <t>9876500001</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -514,29 +514,29 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Mumbai</t>
+          <t>12 Lotus Enclave, Mumbai</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Arjun Patel</t>
+          <t>Ananya Patel</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>arjun.patel@student.edu</t>
+          <t>ananya.patel@student.smartuniversity.edu</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>9876543211</t>
+          <t>9876500002</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Computer Science</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -557,24 +557,24 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>45 Green Park, Pune</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Sneha Gupta</t>
+          <t>Ishaan Verma</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>sneha.gupta@student.edu</t>
+          <t>ishaan.verma@student.smartuniversity.edu</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>9876543212</t>
+          <t>9876500003</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -595,39 +595,39 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Anil Gupta</t>
+          <t>Mahesh Verma</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Delhi</t>
+          <t>88 Civil Lines, Delhi</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rahul Verma</t>
+          <t>Riya Gupta</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>rahul.verma@student.edu</t>
+          <t>riya.gupta@student.smartuniversity.edu</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>9876543213</t>
+          <t>9876500004</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Electronics</t>
+          <t>Computer Science</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>MTech</t>
+          <t>MCA</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -638,34 +638,34 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Rakesh Verma</t>
+          <t>Alok Gupta</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Kolkata</t>
+          <t>77 Ring Road, Bangalore</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Meera Nair</t>
+          <t>Vihaan Das</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>meera.nair@student.edu</t>
+          <t>vihaan.das@student.smartuniversity.edu</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>9876543214</t>
+          <t>9876500005</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Computer Science</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -681,12 +681,141 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Krishna Nair</t>
+          <t>Biplab Das</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Kochi</t>
+          <t>19 Lake View, Kolkata</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Saanvi Iyer</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>saanvi.iyer@student.smartuniversity.edu</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>9876500006</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Computer Science</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>MCA</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Sundar Iyer</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>34 Temple Street, Chennai</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Kabir Mehta</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>kabir.mehta@student.smartuniversity.edu</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>9876500007</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Computer Science</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>MCA</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Nitin Mehta</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>50 University Road, Ahmedabad</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Pooja Reddy</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>pooja.reddy@student.smartuniversity.edu</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>9876500008</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Computer Science</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>MCA</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Venkatesh Reddy</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>22 Hitech City, Hyderabad</t>
         </is>
       </c>
     </row>

</xml_diff>